<commit_message>
feat: análisis completo v8.3 — 17 figuras, sub-período, robustez C4, doc actualizada
- Añade analysis/subperiod.py: análisis laborables vs fines de semana
- Añade fig11_sensibilidad_pgs, fig16_subperiod, fig17_robustez_c4
- Amplía comparison_engine.py: desglose flujos y descomposición bienestar
- Amplía main_simulation.py: modo --full con etiquetas de facturación mensual
- Amplía visualization/plots.py: 17 figuras automáticas
- Amplía feasibility.py: FA-1b IR individual por agente
- Actualiza .gitignore: excluye MedicionesMTE/ y Documentos/
- Actualiza REPORTE_AVANCES.md: estado actual, estructura repo, serie XM confirmada
</commit_message>
<xml_diff>
--- a/resultados_analisis.xlsx
+++ b/resultados_analisis.xlsx
@@ -13,6 +13,8 @@
     <sheet name="Umbrales" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="FA_DesercionIR" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="DesercionIR_Sensibilidad" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="FA3_Robustez_Retiro" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="FA4_Robustez_Escala" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -490,31 +492,31 @@
         <v>200</v>
       </c>
       <c r="B2" t="n">
-        <v>-0.1898421814736614</v>
+        <v>0.1510131705234475</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1710605239449209</v>
+        <v>0.1590835429219084</v>
       </c>
       <c r="D2" t="n">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="E2" t="n">
-        <v>36.62502460436679</v>
+        <v>54.61405283454797</v>
       </c>
       <c r="F2" t="n">
-        <v>135659.3450661442</v>
+        <v>154486.9024422639</v>
       </c>
       <c r="G2" t="n">
-        <v>141744.3515549189</v>
+        <v>165409.7130091735</v>
       </c>
       <c r="H2" t="n">
-        <v>108052.7621285113</v>
+        <v>140833.3892336269</v>
       </c>
       <c r="I2" t="n">
-        <v>108052.7621285113</v>
+        <v>140833.3892336269</v>
       </c>
       <c r="J2" t="n">
-        <v>112453.3864211047</v>
+        <v>129910.5786667173</v>
       </c>
     </row>
     <row r="3">
@@ -522,31 +524,31 @@
         <v>250</v>
       </c>
       <c r="B3" t="n">
-        <v>-0.1898421814736614</v>
+        <v>0.1510131705234475</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1436078622832272</v>
+        <v>0.1439520834241526</v>
       </c>
       <c r="D3" t="n">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="E3" t="n">
-        <v>36.62502460436679</v>
+        <v>54.61405283454797</v>
       </c>
       <c r="F3" t="n">
-        <v>133828.0938359258</v>
+        <v>151756.1998005365</v>
       </c>
       <c r="G3" t="n">
-        <v>142852.4133778994</v>
+        <v>165409.7130091735</v>
       </c>
       <c r="H3" t="n">
-        <v>110765.1853527494</v>
+        <v>143564.0918753543</v>
       </c>
       <c r="I3" t="n">
-        <v>110765.1853527494</v>
+        <v>143564.0918753543</v>
       </c>
       <c r="J3" t="n">
-        <v>114609.3273667094</v>
+        <v>129910.5786667173</v>
       </c>
     </row>
     <row r="4">
@@ -554,31 +556,31 @@
         <v>280</v>
       </c>
       <c r="B4" t="n">
-        <v>-0.1898421814736614</v>
+        <v>0.1510131705234475</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1267726545691174</v>
+        <v>0.1346089702964729</v>
       </c>
       <c r="D4" t="n">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="E4" t="n">
-        <v>36.62502460436679</v>
+        <v>54.61405283454797</v>
       </c>
       <c r="F4" t="n">
-        <v>132729.3430977948</v>
+        <v>150117.7782155001</v>
       </c>
       <c r="G4" t="n">
-        <v>143517.2504716878</v>
+        <v>165409.7130091735</v>
       </c>
       <c r="H4" t="n">
-        <v>112392.6392872922</v>
+        <v>145202.5134603907</v>
       </c>
       <c r="I4" t="n">
-        <v>112392.6392872922</v>
+        <v>145202.5134603907</v>
       </c>
       <c r="J4" t="n">
-        <v>115902.8919340722</v>
+        <v>129910.5786667173</v>
       </c>
     </row>
     <row r="5">
@@ -586,31 +588,31 @@
         <v>300</v>
       </c>
       <c r="B5" t="n">
-        <v>-0.1898421814736614</v>
+        <v>0.1510131705234475</v>
       </c>
       <c r="C5" t="n">
-        <v>0.1153934745158426</v>
+        <v>0.128266094436994</v>
       </c>
       <c r="D5" t="n">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="E5" t="n">
-        <v>36.62502460436679</v>
+        <v>54.61405283454797</v>
       </c>
       <c r="F5" t="n">
-        <v>131996.8426057075</v>
+        <v>149025.4971588091</v>
       </c>
       <c r="G5" t="n">
-        <v>143960.47520088</v>
+        <v>165409.7130091735</v>
       </c>
       <c r="H5" t="n">
-        <v>113477.6085769874</v>
+        <v>146294.7945170817</v>
       </c>
       <c r="I5" t="n">
-        <v>113477.6085769874</v>
+        <v>146294.7945170817</v>
       </c>
       <c r="J5" t="n">
-        <v>116765.2683123141</v>
+        <v>129910.5786667173</v>
       </c>
     </row>
     <row r="6">
@@ -618,31 +620,31 @@
         <v>350</v>
       </c>
       <c r="B6" t="n">
-        <v>-0.1898421814736614</v>
+        <v>0.1510131705234475</v>
       </c>
       <c r="C6" t="n">
-        <v>0.08638521132004615</v>
+        <v>0.111994523827376</v>
       </c>
       <c r="D6" t="n">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="E6" t="n">
-        <v>36.62502460436679</v>
+        <v>54.61405283454797</v>
       </c>
       <c r="F6" t="n">
-        <v>130165.5913754892</v>
+        <v>146294.7945170817</v>
       </c>
       <c r="G6" t="n">
-        <v>145068.5370238606</v>
+        <v>165409.7130091735</v>
       </c>
       <c r="H6" t="n">
-        <v>116190.0318012255</v>
+        <v>149025.4971588091</v>
       </c>
       <c r="I6" t="n">
-        <v>116190.0318012255</v>
+        <v>149025.4971588091</v>
       </c>
       <c r="J6" t="n">
-        <v>118921.2092579187</v>
+        <v>129910.5786667173</v>
       </c>
     </row>
     <row r="7">
@@ -650,31 +652,31 @@
         <v>400</v>
       </c>
       <c r="B7" t="n">
-        <v>-0.1898421814736614</v>
+        <v>0.1510131705234475</v>
       </c>
       <c r="C7" t="n">
-        <v>0.05654908836974167</v>
+        <v>0.09510395691766214</v>
       </c>
       <c r="D7" t="n">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="E7" t="n">
-        <v>36.62502460436679</v>
+        <v>54.61405283454797</v>
       </c>
       <c r="F7" t="n">
-        <v>128334.3401452708</v>
+        <v>143564.0918753543</v>
       </c>
       <c r="G7" t="n">
-        <v>146176.5988468411</v>
+        <v>165409.7130091735</v>
       </c>
       <c r="H7" t="n">
-        <v>118902.4550254635</v>
+        <v>151756.1998005365</v>
       </c>
       <c r="I7" t="n">
-        <v>118902.4550254635</v>
+        <v>151756.1998005365</v>
       </c>
       <c r="J7" t="n">
-        <v>121077.1502035234</v>
+        <v>129910.5786667173</v>
       </c>
     </row>
     <row r="8">
@@ -682,31 +684,31 @@
         <v>450</v>
       </c>
       <c r="B8" t="n">
-        <v>-0.1898421814736614</v>
+        <v>0.1510131705234475</v>
       </c>
       <c r="C8" t="n">
-        <v>0.02584915351845844</v>
+        <v>0.07755838744170146</v>
       </c>
       <c r="D8" t="n">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="E8" t="n">
-        <v>36.62502460436679</v>
+        <v>54.61405283454797</v>
       </c>
       <c r="F8" t="n">
-        <v>126503.0889150525</v>
+        <v>140833.3892336269</v>
       </c>
       <c r="G8" t="n">
-        <v>147284.6606698217</v>
+        <v>165409.7130091735</v>
       </c>
       <c r="H8" t="n">
-        <v>121614.8782497016</v>
+        <v>154486.9024422639</v>
       </c>
       <c r="I8" t="n">
-        <v>121614.8782497016</v>
+        <v>154486.9024422639</v>
       </c>
       <c r="J8" t="n">
-        <v>123233.0911491281</v>
+        <v>129910.5786667173</v>
       </c>
     </row>
     <row r="9">
@@ -714,31 +716,31 @@
         <v>500</v>
       </c>
       <c r="B9" t="n">
-        <v>-0.1898421814736614</v>
+        <v>0.1510131705234475</v>
       </c>
       <c r="C9" t="n">
-        <v>-0.005752657723002806</v>
+        <v>0.05931896132759733</v>
       </c>
       <c r="D9" t="n">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="E9" t="n">
-        <v>36.62502460436679</v>
+        <v>54.61405283454797</v>
       </c>
       <c r="F9" t="n">
-        <v>124671.8376848341</v>
+        <v>138102.6865918995</v>
       </c>
       <c r="G9" t="n">
-        <v>148392.7224928022</v>
+        <v>165409.7130091735</v>
       </c>
       <c r="H9" t="n">
-        <v>124327.3014739396</v>
+        <v>157217.6050839913</v>
       </c>
       <c r="I9" t="n">
-        <v>124327.3014739396</v>
+        <v>157217.6050839913</v>
       </c>
       <c r="J9" t="n">
-        <v>125389.0320947327</v>
+        <v>129910.5786667173</v>
       </c>
     </row>
   </sheetData>
@@ -752,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -810,25 +812,170 @@
         <v>11.3</v>
       </c>
       <c r="C2" t="n">
-        <v>-0.1898421814736614</v>
+        <v>0.1510131705234475</v>
       </c>
       <c r="D2" t="n">
-        <v>0.8665001357634031</v>
+        <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="F2" t="n">
-        <v>36.62502460436679</v>
+        <v>54.61405283454797</v>
       </c>
       <c r="G2" t="n">
-        <v>138809.0971821197</v>
+        <v>150117.7782155001</v>
       </c>
       <c r="H2" t="n">
-        <v>139838.4852193923</v>
+        <v>165409.7130091735</v>
       </c>
       <c r="I2" t="n">
-        <v>108745.1679946647</v>
+        <v>129910.5786667173</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1.775059274451622</v>
+      </c>
+      <c r="B3" t="n">
+        <v>20.05816980130333</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.08922019760959191</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F3" t="n">
+        <v>120.4285240481381</v>
+      </c>
+      <c r="G3" t="n">
+        <v>259892.0584278358</v>
+      </c>
+      <c r="H3" t="n">
+        <v>293612.0451613145</v>
+      </c>
+      <c r="I3" t="n">
+        <v>215333.5045300248</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2.928847802845176</v>
+      </c>
+      <c r="B4" t="n">
+        <v>33.09598017215049</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.4750296754428208</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.9607029465548876</v>
+      </c>
+      <c r="E4" t="n">
+        <v>10</v>
+      </c>
+      <c r="F4" t="n">
+        <v>223.8495887595365</v>
+      </c>
+      <c r="G4" t="n">
+        <v>402744.1440826245</v>
+      </c>
+      <c r="H4" t="n">
+        <v>448678.5715493655</v>
+      </c>
+      <c r="I4" t="n">
+        <v>350316.8441996673</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4.437648186129055</v>
+      </c>
+      <c r="B5" t="n">
+        <v>50.14542450325832</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.7059157606489921</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.7826120834016972</v>
+      </c>
+      <c r="E5" t="n">
+        <v>10</v>
+      </c>
+      <c r="F5" t="n">
+        <v>245.285790267327</v>
+      </c>
+      <c r="G5" t="n">
+        <v>505780.8146639722</v>
+      </c>
+      <c r="H5" t="n">
+        <v>645337.1065262257</v>
+      </c>
+      <c r="I5" t="n">
+        <v>566073.86680205</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>6.656472279193582</v>
+      </c>
+      <c r="B6" t="n">
+        <v>75.21813675488748</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.8712738080296112</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.5899925144493797</v>
+      </c>
+      <c r="E6" t="n">
+        <v>9</v>
+      </c>
+      <c r="F6" t="n">
+        <v>195.1953866282991</v>
+      </c>
+      <c r="G6" t="n">
+        <v>594953.6997341341</v>
+      </c>
+      <c r="H6" t="n">
+        <v>934540.8344333732</v>
+      </c>
+      <c r="I6" t="n">
+        <v>812628.8914254026</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>8.875296372258109</v>
+      </c>
+      <c r="B7" t="n">
+        <v>100.2908490065166</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.8764198774039593</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.4673136919147121</v>
+      </c>
+      <c r="E7" t="n">
+        <v>8</v>
+      </c>
+      <c r="F7" t="n">
+        <v>136.885324931328</v>
+      </c>
+      <c r="G7" t="n">
+        <v>647716.7530940431</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1206826.278348739</v>
+      </c>
+      <c r="I7" t="n">
+        <v>989477.6634026923</v>
       </c>
     </row>
   </sheetData>
@@ -842,7 +989,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -880,17 +1027,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>Udenar</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>48.32</v>
+        <v>4.2</v>
       </c>
       <c r="C2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>4</v>
+        <v>12.7</v>
       </c>
       <c r="E2" t="b">
         <v>1</v>
@@ -900,17 +1047,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>Mariana</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>23.46</v>
+        <v>1.88</v>
       </c>
       <c r="C3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>4</v>
+        <v>5.8</v>
       </c>
       <c r="E3" t="b">
         <v>1</v>
@@ -920,17 +1067,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>A3</t>
+          <t>UCC</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>11.26</v>
+        <v>2.36</v>
       </c>
       <c r="C4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D4" t="n">
-        <v>2.5</v>
+        <v>7</v>
       </c>
       <c r="E4" t="b">
         <v>1</v>
@@ -940,17 +1087,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>A4</t>
+          <t>HUDN</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>19.36</v>
+        <v>1.79</v>
       </c>
       <c r="C5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>1.5</v>
+        <v>5.6</v>
       </c>
       <c r="E5" t="b">
         <v>1</v>
@@ -960,17 +1107,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>A5</t>
+          <t>Cesmag</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>1.04</v>
       </c>
       <c r="C6" t="b">
         <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>2.9</v>
       </c>
       <c r="E6" t="b">
         <v>1</v>
@@ -980,35 +1127,15 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>A6</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" t="b">
-        <v>1</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" t="b">
-        <v>1</v>
-      </c>
-      <c r="F7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
           <t>COMUNIDAD</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="n">
-        <v>0.5</v>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1059,10 +1186,12 @@
     </row>
     <row r="2">
       <c r="A2" t="b">
-        <v>0</v>
-      </c>
-      <c r="B2" t="n">
-        <v>491.0062723556762</v>
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>siempre_mejor</t>
+        </is>
       </c>
       <c r="C2" t="b">
         <v>0</v>
@@ -1077,7 +1206,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>{1.0: 24}</t>
+          <t>{1.0: 7, 1.775059274451622: 9, 2.9288478028451763: 10, 4.437648186129055: 10, 6.656472279193582: 9, 8.87529637225811: 8}</t>
         </is>
       </c>
     </row>
@@ -1092,7 +1221,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1135,20 +1264,20 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>Udenar</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>66488.87224966632</v>
+        <v>34243.97455063702</v>
       </c>
       <c r="C2" t="n">
-        <v>68766.10632519744</v>
+        <v>61607.21690378158</v>
       </c>
       <c r="D2" t="n">
-        <v>-2277.234075531116</v>
+        <v>-27363.24235314456</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.03311564660593102</v>
+        <v>-0.4441564434874666</v>
       </c>
       <c r="F2" t="n">
         <v>180</v>
@@ -1162,77 +1291,77 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>Mariana</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>19810.00361875292</v>
+        <v>32297.31385398124</v>
       </c>
       <c r="C3" t="n">
-        <v>22737.72379661772</v>
+        <v>27554.99749148169</v>
       </c>
       <c r="D3" t="n">
-        <v>-2927.720177864801</v>
+        <v>4742.316362499554</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.1287604777000724</v>
+        <v>0.1721036760742071</v>
       </c>
       <c r="F3" t="n">
-        <v>180</v>
+        <v>550</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>en_riesgo</t>
+          <t>estable</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>A3</t>
+          <t>UCC</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>12172.28445731253</v>
+        <v>34678.53872393133</v>
       </c>
       <c r="C4" t="n">
-        <v>15272.55083458049</v>
+        <v>34678.53872393088</v>
       </c>
       <c r="D4" t="n">
-        <v>-3100.266377267953</v>
+        <v>4.43833414465189e-10</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.2029959769554837</v>
+        <v>1.279850393923633e-14</v>
       </c>
       <c r="F4" t="n">
-        <v>180</v>
+        <v>550</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>en_riesgo</t>
+          <t>estable</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>A4</t>
+          <t>HUDN</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>35698.66526948559</v>
+        <v>29463.09716747679</v>
       </c>
       <c r="C5" t="n">
-        <v>33062.10426299669</v>
+        <v>26291.02206540454</v>
       </c>
       <c r="D5" t="n">
-        <v>2636.561006488904</v>
+        <v>3172.075102072253</v>
       </c>
       <c r="E5" t="n">
-        <v>0.07974571084514301</v>
+        <v>0.1206524072811258</v>
       </c>
       <c r="F5" t="n">
-        <v>449.3</v>
+        <v>550</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -1243,52 +1372,25 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>A5</t>
+          <t>Cesmag</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2568.91097435111</v>
+        <v>19434.85391947367</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>15277.93782457481</v>
       </c>
       <c r="D6" t="n">
-        <v>2568.91097435111</v>
+        <v>4156.916094898859</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>0.2720862031662671</v>
       </c>
       <c r="F6" t="n">
         <v>550</v>
       </c>
       <c r="G6" t="inlineStr">
-        <is>
-          <t>estable</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>A6</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>2070.360612551229</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" t="n">
-        <v>2070.360612551229</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" t="n">
-        <v>550</v>
-      </c>
-      <c r="G7" t="inlineStr">
         <is>
           <t>estable</t>
         </is>
@@ -1305,7 +1407,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1316,35 +1418,30 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>delta_A1</t>
+          <t>delta_Udenar</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>delta_A2</t>
+          <t>delta_Mariana</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>delta_A3</t>
+          <t>delta_UCC</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>delta_A4</t>
+          <t>delta_HUDN</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>delta_A5</t>
+          <t>delta_Cesmag</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>delta_A6</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>delta_total</t>
         </is>
@@ -1355,25 +1452,22 @@
         <v>200</v>
       </c>
       <c r="B2" t="n">
-        <v>-2970.036433874251</v>
+        <v>-22994.11812638072</v>
       </c>
       <c r="C2" t="n">
-        <v>-5573.547826432747</v>
+        <v>4742.316362499554</v>
       </c>
       <c r="D2" t="n">
-        <v>-4140.940938408503</v>
+        <v>4.43833414465189e-10</v>
       </c>
       <c r="E2" t="n">
-        <v>1960.24712303844</v>
+        <v>3172.075102072253</v>
       </c>
       <c r="F2" t="n">
-        <v>2568.91097435111</v>
+        <v>4156.916094898859</v>
       </c>
       <c r="G2" t="n">
-        <v>2070.360612551229</v>
-      </c>
-      <c r="H2" t="n">
-        <v>-6085.006488774721</v>
+        <v>-10922.81056690961</v>
       </c>
     </row>
     <row r="3">
@@ -1381,25 +1475,22 @@
         <v>250</v>
       </c>
       <c r="B3" t="n">
-        <v>-3372.8285026784</v>
+        <v>-25724.82076810812</v>
       </c>
       <c r="C3" t="n">
-        <v>-7111.819715135036</v>
+        <v>4742.316362499554</v>
       </c>
       <c r="D3" t="n">
-        <v>-4745.984287908825</v>
+        <v>4.43833414465189e-10</v>
       </c>
       <c r="E3" t="n">
-        <v>1567.041376846304</v>
+        <v>3172.075102072253</v>
       </c>
       <c r="F3" t="n">
-        <v>2568.91097435111</v>
+        <v>4156.916094898859</v>
       </c>
       <c r="G3" t="n">
-        <v>2070.360612551229</v>
-      </c>
-      <c r="H3" t="n">
-        <v>-9024.319541973617</v>
+        <v>-13653.51320863701</v>
       </c>
     </row>
     <row r="4">
@@ -1407,25 +1498,22 @@
         <v>280</v>
       </c>
       <c r="B4" t="n">
-        <v>-3614.5037439609</v>
+        <v>-27363.24235314456</v>
       </c>
       <c r="C4" t="n">
-        <v>-8034.782848356412</v>
+        <v>4742.316362499554</v>
       </c>
       <c r="D4" t="n">
-        <v>-5109.010297609018</v>
+        <v>4.43833414465189e-10</v>
       </c>
       <c r="E4" t="n">
-        <v>1331.117929131025</v>
+        <v>3172.075102072253</v>
       </c>
       <c r="F4" t="n">
-        <v>2568.91097435111</v>
+        <v>4156.916094898859</v>
       </c>
       <c r="G4" t="n">
-        <v>2070.360612551229</v>
-      </c>
-      <c r="H4" t="n">
-        <v>-10787.90737389297</v>
+        <v>-15291.93479367345</v>
       </c>
     </row>
     <row r="5">
@@ -1433,25 +1521,22 @@
         <v>300</v>
       </c>
       <c r="B5" t="n">
-        <v>-3775.620571482563</v>
+        <v>-28455.52340983552</v>
       </c>
       <c r="C5" t="n">
-        <v>-8650.091603837329</v>
+        <v>4742.316362499554</v>
       </c>
       <c r="D5" t="n">
-        <v>-5351.027637409145</v>
+        <v>4.43833414465189e-10</v>
       </c>
       <c r="E5" t="n">
-        <v>1173.835630654175</v>
+        <v>3172.075102072253</v>
       </c>
       <c r="F5" t="n">
-        <v>2568.91097435111</v>
+        <v>4156.916094898859</v>
       </c>
       <c r="G5" t="n">
-        <v>2070.360612551229</v>
-      </c>
-      <c r="H5" t="n">
-        <v>-11963.63259517252</v>
+        <v>-16384.21585036441</v>
       </c>
     </row>
     <row r="6">
@@ -1459,25 +1544,22 @@
         <v>350</v>
       </c>
       <c r="B6" t="n">
-        <v>-4178.412640286704</v>
+        <v>-31186.22605156291</v>
       </c>
       <c r="C6" t="n">
-        <v>-10188.36349253962</v>
+        <v>4742.316362499554</v>
       </c>
       <c r="D6" t="n">
-        <v>-5956.070986909466</v>
+        <v>4.43833414465189e-10</v>
       </c>
       <c r="E6" t="n">
-        <v>780.6298844620396</v>
+        <v>3172.075102072253</v>
       </c>
       <c r="F6" t="n">
-        <v>2568.91097435111</v>
+        <v>4156.916094898859</v>
       </c>
       <c r="G6" t="n">
-        <v>2070.360612551229</v>
-      </c>
-      <c r="H6" t="n">
-        <v>-14902.94564837141</v>
+        <v>-19114.91849209181</v>
       </c>
     </row>
     <row r="7">
@@ -1485,25 +1567,22 @@
         <v>400</v>
       </c>
       <c r="B7" t="n">
-        <v>-4581.204709090853</v>
+        <v>-33916.92869329031</v>
       </c>
       <c r="C7" t="n">
-        <v>-11726.63538124191</v>
+        <v>4742.316362499554</v>
       </c>
       <c r="D7" t="n">
-        <v>-6561.114336409788</v>
+        <v>4.43833414465189e-10</v>
       </c>
       <c r="E7" t="n">
-        <v>387.4241382699038</v>
+        <v>3172.075102072253</v>
       </c>
       <c r="F7" t="n">
-        <v>2568.91097435111</v>
+        <v>4156.916094898859</v>
       </c>
       <c r="G7" t="n">
-        <v>2070.360612551229</v>
-      </c>
-      <c r="H7" t="n">
-        <v>-17842.25870157031</v>
+        <v>-21845.62113381919</v>
       </c>
     </row>
     <row r="8">
@@ -1511,25 +1590,22 @@
         <v>450</v>
       </c>
       <c r="B8" t="n">
-        <v>-4983.996777894994</v>
+        <v>-36647.63133501771</v>
       </c>
       <c r="C8" t="n">
-        <v>-13264.90726994421</v>
+        <v>4742.316362499554</v>
       </c>
       <c r="D8" t="n">
-        <v>-7166.15768591011</v>
+        <v>4.43833414465189e-10</v>
       </c>
       <c r="E8" t="n">
-        <v>-5.78160792223207</v>
+        <v>3172.075102072253</v>
       </c>
       <c r="F8" t="n">
-        <v>2568.91097435111</v>
+        <v>4156.916094898859</v>
       </c>
       <c r="G8" t="n">
-        <v>2070.360612551229</v>
-      </c>
-      <c r="H8" t="n">
-        <v>-20781.57175476921</v>
+        <v>-24576.3237755466</v>
       </c>
     </row>
     <row r="9">
@@ -1537,25 +1613,424 @@
         <v>500</v>
       </c>
       <c r="B9" t="n">
-        <v>-5386.788846699143</v>
+        <v>-39378.33397674511</v>
       </c>
       <c r="C9" t="n">
-        <v>-14803.1791586465</v>
+        <v>4742.316362499554</v>
       </c>
       <c r="D9" t="n">
-        <v>-7771.20103541043</v>
+        <v>4.43833414465189e-10</v>
       </c>
       <c r="E9" t="n">
-        <v>-398.9873541143606</v>
+        <v>3172.075102072253</v>
       </c>
       <c r="F9" t="n">
-        <v>2568.91097435111</v>
+        <v>4156.916094898859</v>
       </c>
       <c r="G9" t="n">
-        <v>2070.360612551229</v>
-      </c>
-      <c r="H9" t="n">
-        <v>-23720.88480796809</v>
+        <v>-27307.026417274</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Agente_retirado</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>AGRC_restante_cumple</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>B_C4_full_COP</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>B_C4_remaining_COP</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>B_fallback_COP</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>B_P2P_remaining_COP</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>loss_C4_COP</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>flexibility_premium_COP</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>reglas_violadas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Udenar</t>
+        </is>
+      </c>
+      <c r="B2" t="b">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>129910.5786667173</v>
+      </c>
+      <c r="D2" t="n">
+        <v>103802.4961053919</v>
+      </c>
+      <c r="E2" t="n">
+        <v>103802.4961053919</v>
+      </c>
+      <c r="F2" t="n">
+        <v>115873.803664863</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>12071.30755947111</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Mariana</t>
+        </is>
+      </c>
+      <c r="B3" t="b">
+        <v>1</v>
+      </c>
+      <c r="C3" t="n">
+        <v>129910.5786667173</v>
+      </c>
+      <c r="D3" t="n">
+        <v>102355.5811752356</v>
+      </c>
+      <c r="E3" t="n">
+        <v>102355.5811752356</v>
+      </c>
+      <c r="F3" t="n">
+        <v>117820.4643615188</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>15464.88318628317</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>UCC</t>
+        </is>
+      </c>
+      <c r="B4" t="b">
+        <v>1</v>
+      </c>
+      <c r="C4" t="n">
+        <v>129910.5786667173</v>
+      </c>
+      <c r="D4" t="n">
+        <v>95232.03994278643</v>
+      </c>
+      <c r="E4" t="n">
+        <v>95232.03994278643</v>
+      </c>
+      <c r="F4" t="n">
+        <v>115439.2394915687</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>20207.1995487823</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>HUDN</t>
+        </is>
+      </c>
+      <c r="B5" t="b">
+        <v>1</v>
+      </c>
+      <c r="C5" t="n">
+        <v>129910.5786667173</v>
+      </c>
+      <c r="D5" t="n">
+        <v>103619.5566013128</v>
+      </c>
+      <c r="E5" t="n">
+        <v>103619.5566013128</v>
+      </c>
+      <c r="F5" t="n">
+        <v>120654.6810480233</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>17035.12444671048</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Cesmag</t>
+        </is>
+      </c>
+      <c r="B6" t="b">
+        <v>1</v>
+      </c>
+      <c r="C6" t="n">
+        <v>129910.5786667173</v>
+      </c>
+      <c r="D6" t="n">
+        <v>114632.6408421425</v>
+      </c>
+      <c r="E6" t="n">
+        <v>114632.6408421425</v>
+      </c>
+      <c r="F6" t="n">
+        <v>130682.9242960264</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>16050.28345388388</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Agente</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>G_mean_kW</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>G_max_kW</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Share_actual_%</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>2x_cumple</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>3x_cumple</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Escala_max_ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Udenar</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="C2" t="n">
+        <v>12.69</v>
+      </c>
+      <c r="D2" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Mariana</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="C3" t="n">
+        <v>5.83</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="E3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>UCC</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="C4" t="n">
+        <v>7.03</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="E4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F4" t="b">
+        <v>1</v>
+      </c>
+      <c r="G4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>HUDN</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="C5" t="n">
+        <v>5.59</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="E5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G5" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Cesmag</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="C6" t="n">
+        <v>2.94</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="E6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F6" t="b">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>